<commit_message>
Daily NSE scan: 2026-10-07
</commit_message>
<xml_diff>
--- a/output/2026-10-07/enriched_analysis.xlsx
+++ b/output/2026-10-07/enriched_analysis.xlsx
@@ -929,13 +929,13 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>2.188</v>
+        <v>2.062</v>
       </c>
       <c r="W2" t="n">
-        <v>2880</v>
+        <v>3056</v>
       </c>
       <c r="X2" t="n">
-        <v>22.6</v>
+        <v>23.9</v>
       </c>
       <c r="Y2" t="n">
         <v>75</v>
@@ -1161,10 +1161,10 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>0.843</v>
+        <v>0.845</v>
       </c>
       <c r="W3" t="n">
-        <v>960</v>
+        <v>958</v>
       </c>
       <c r="X3" t="n">
         <v>134</v>
@@ -1393,13 +1393,13 @@
         </is>
       </c>
       <c r="V4" t="n">
-        <v>0.048</v>
+        <v>0.047</v>
       </c>
       <c r="W4" t="n">
-        <v>2765</v>
+        <v>2836</v>
       </c>
       <c r="X4" t="n">
-        <v>9.5</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="Y4" t="n">
         <v>36</v>
@@ -1625,13 +1625,13 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>1.162</v>
+        <v>1.166</v>
       </c>
       <c r="W5" t="n">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="X5" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="Y5" t="n">
         <v>22</v>
@@ -1857,10 +1857,10 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>1.707</v>
+        <v>1.742</v>
       </c>
       <c r="W6" t="n">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="n">
@@ -2087,13 +2087,13 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>0.325</v>
+        <v>0.323</v>
       </c>
       <c r="W7" t="n">
-        <v>942</v>
+        <v>948</v>
       </c>
       <c r="X7" t="n">
-        <v>9.26</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="Y7" t="n">
         <v>7</v>
@@ -2319,13 +2319,13 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>0.53</v>
+        <v>0.537</v>
       </c>
       <c r="W8" t="n">
-        <v>2696</v>
+        <v>2660</v>
       </c>
       <c r="X8" t="n">
-        <v>22.1</v>
+        <v>21.8</v>
       </c>
       <c r="Y8" t="n">
         <v>8</v>
@@ -2557,7 +2557,7 @@
         <v>185</v>
       </c>
       <c r="X9" t="n">
-        <v>7.86</v>
+        <v>7.87</v>
       </c>
       <c r="Y9" t="n">
         <v>17</v>
@@ -2783,13 +2783,13 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>0.049</v>
+        <v>0.048</v>
       </c>
       <c r="W10" t="n">
-        <v>14790</v>
+        <v>15093</v>
       </c>
       <c r="X10" t="n">
-        <v>37.7</v>
+        <v>38.5</v>
       </c>
       <c r="Y10" t="n">
         <v>83</v>
@@ -3018,7 +3018,7 @@
         <v>0.126</v>
       </c>
       <c r="W11" t="n">
-        <v>2483</v>
+        <v>2484</v>
       </c>
       <c r="X11" t="n">
         <v>21.8</v>
@@ -3247,10 +3247,10 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>2.254</v>
+        <v>2.261</v>
       </c>
       <c r="W12" t="n">
-        <v>2604</v>
+        <v>2596</v>
       </c>
       <c r="X12" t="n">
         <v>204</v>
@@ -3482,10 +3482,10 @@
         <v>0.048</v>
       </c>
       <c r="W13" t="n">
-        <v>1718</v>
+        <v>1704</v>
       </c>
       <c r="X13" t="n">
-        <v>23.1</v>
+        <v>22.9</v>
       </c>
       <c r="Y13" t="n">
         <v>55</v>
@@ -3711,13 +3711,13 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>0.065</v>
+        <v>0.066</v>
       </c>
       <c r="W14" t="n">
-        <v>874</v>
+        <v>862</v>
       </c>
       <c r="X14" t="n">
-        <v>22.1</v>
+        <v>21.8</v>
       </c>
       <c r="Y14" t="n">
         <v>19</v>
@@ -3941,13 +3941,13 @@
         </is>
       </c>
       <c r="V15" t="n">
-        <v>2.714</v>
+        <v>2.783</v>
       </c>
       <c r="W15" t="n">
-        <v>725</v>
+        <v>707</v>
       </c>
       <c r="X15" t="n">
-        <v>21.9</v>
+        <v>21.4</v>
       </c>
       <c r="Y15" t="n">
         <v>30</v>
@@ -4167,13 +4167,13 @@
         </is>
       </c>
       <c r="V16" t="n">
-        <v>0.063</v>
+        <v>0.064</v>
       </c>
       <c r="W16" t="n">
-        <v>1746</v>
+        <v>1727</v>
       </c>
       <c r="X16" t="n">
-        <v>40.1</v>
+        <v>39.7</v>
       </c>
       <c r="Y16" t="n">
         <v>20</v>
@@ -4399,13 +4399,13 @@
         </is>
       </c>
       <c r="V17" t="n">
-        <v>0.123</v>
+        <v>0.12</v>
       </c>
       <c r="W17" t="n">
-        <v>700</v>
+        <v>716</v>
       </c>
       <c r="X17" t="n">
-        <v>30.5</v>
+        <v>31.2</v>
       </c>
       <c r="Y17" t="n">
         <v>17</v>
@@ -4625,10 +4625,10 @@
         </is>
       </c>
       <c r="V18" t="n">
-        <v>1.814</v>
+        <v>1.845</v>
       </c>
       <c r="W18" t="n">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="X18" t="inlineStr"/>
       <c r="Y18" t="n">
@@ -4858,10 +4858,10 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="W19" t="n">
-        <v>55099</v>
+        <v>54470</v>
       </c>
       <c r="X19" t="n">
-        <v>46.7</v>
+        <v>46.2</v>
       </c>
       <c r="Y19" t="n">
         <v>5</v>
@@ -5087,13 +5087,13 @@
         </is>
       </c>
       <c r="V20" t="n">
-        <v>0.185</v>
+        <v>0.179</v>
       </c>
       <c r="W20" t="n">
-        <v>600</v>
+        <v>619</v>
       </c>
       <c r="X20" t="n">
-        <v>50.1</v>
+        <v>51.7</v>
       </c>
       <c r="Y20" t="n">
         <v>3</v>
@@ -5319,13 +5319,13 @@
         </is>
       </c>
       <c r="V21" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.089</v>
       </c>
       <c r="W21" t="n">
-        <v>657</v>
+        <v>644</v>
       </c>
       <c r="X21" t="n">
-        <v>10.7</v>
+        <v>10.5</v>
       </c>
       <c r="Y21" t="n">
         <v>-5</v>
@@ -5551,13 +5551,13 @@
         </is>
       </c>
       <c r="V22" t="n">
-        <v>0.37</v>
+        <v>0.369</v>
       </c>
       <c r="W22" t="n">
-        <v>1063</v>
+        <v>1067</v>
       </c>
       <c r="X22" t="n">
-        <v>54.2</v>
+        <v>54.3</v>
       </c>
       <c r="Y22" t="n">
         <v>21</v>
@@ -5783,13 +5783,13 @@
         </is>
       </c>
       <c r="V23" t="n">
-        <v>0.663</v>
+        <v>0.679</v>
       </c>
       <c r="W23" t="n">
-        <v>437</v>
+        <v>427</v>
       </c>
       <c r="X23" t="n">
-        <v>10.9</v>
+        <v>10.7</v>
       </c>
       <c r="Y23" t="n">
         <v>19</v>
@@ -6015,13 +6015,13 @@
         </is>
       </c>
       <c r="V24" t="n">
-        <v>1.033</v>
+        <v>1.012</v>
       </c>
       <c r="W24" t="n">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="X24" t="n">
-        <v>5.63</v>
+        <v>5.73</v>
       </c>
       <c r="Y24" t="n">
         <v>31</v>
@@ -6243,13 +6243,13 @@
         </is>
       </c>
       <c r="V25" t="n">
-        <v>0.328</v>
+        <v>0.347</v>
       </c>
       <c r="W25" t="n">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="X25" t="n">
-        <v>23.4</v>
+        <v>22.1</v>
       </c>
       <c r="Y25" t="n">
         <v>12</v>
@@ -6475,13 +6475,13 @@
         </is>
       </c>
       <c r="V26" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
       <c r="W26" t="n">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="X26" t="n">
-        <v>36.1</v>
+        <v>35.7</v>
       </c>
       <c r="Y26" t="n">
         <v>21</v>
@@ -6707,13 +6707,13 @@
         </is>
       </c>
       <c r="V27" t="n">
-        <v>0.519</v>
+        <v>0.516</v>
       </c>
       <c r="W27" t="n">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="X27" t="n">
-        <v>35.9</v>
+        <v>36</v>
       </c>
       <c r="Y27" t="n">
         <v>-44</v>
@@ -6939,13 +6939,13 @@
         </is>
       </c>
       <c r="V28" t="n">
-        <v>0.136</v>
+        <v>0.125</v>
       </c>
       <c r="W28" t="n">
-        <v>588</v>
+        <v>641</v>
       </c>
       <c r="X28" t="n">
-        <v>13</v>
+        <v>14.1</v>
       </c>
       <c r="Y28" t="n">
         <v>-1</v>
@@ -7171,13 +7171,13 @@
         </is>
       </c>
       <c r="V29" t="n">
-        <v>0.237</v>
+        <v>0.235</v>
       </c>
       <c r="W29" t="n">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="X29" t="n">
-        <v>14.4</v>
+        <v>14.5</v>
       </c>
       <c r="Y29" t="n">
         <v>16</v>
@@ -7406,7 +7406,7 @@
         <v>0.043</v>
       </c>
       <c r="W30" t="n">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="X30" t="n">
         <v>20.9</v>
@@ -7861,13 +7861,13 @@
         </is>
       </c>
       <c r="V32" t="n">
-        <v>0.829</v>
+        <v>0.819</v>
       </c>
       <c r="W32" t="n">
-        <v>3810</v>
+        <v>3856</v>
       </c>
       <c r="X32" t="n">
-        <v>26.7</v>
+        <v>27</v>
       </c>
       <c r="Y32" t="n">
         <v>2</v>
@@ -8093,13 +8093,13 @@
         </is>
       </c>
       <c r="V33" t="n">
-        <v>0.291</v>
+        <v>0.283</v>
       </c>
       <c r="W33" t="n">
-        <v>895</v>
+        <v>919</v>
       </c>
       <c r="X33" t="n">
-        <v>24.4</v>
+        <v>25</v>
       </c>
       <c r="Y33" t="n">
         <v>9</v>
@@ -8325,13 +8325,13 @@
         </is>
       </c>
       <c r="V34" t="n">
-        <v>0.663</v>
+        <v>0.671</v>
       </c>
       <c r="W34" t="n">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="X34" t="n">
-        <v>1142</v>
+        <v>1130</v>
       </c>
       <c r="Y34" t="n">
         <v>-61</v>
@@ -8559,7 +8559,7 @@
         <v>384</v>
       </c>
       <c r="X35" t="n">
-        <v>95</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="Y35" t="n">
         <v>246</v>
@@ -8785,13 +8785,13 @@
         </is>
       </c>
       <c r="V36" t="n">
-        <v>0.226</v>
+        <v>0.228</v>
       </c>
       <c r="W36" t="n">
-        <v>1766</v>
+        <v>1752</v>
       </c>
       <c r="X36" t="n">
-        <v>18.7</v>
+        <v>18.6</v>
       </c>
       <c r="Y36" t="n">
         <v>-3</v>
@@ -9020,10 +9020,10 @@
         <v>0.041</v>
       </c>
       <c r="W37" t="n">
-        <v>3257</v>
+        <v>3275</v>
       </c>
       <c r="X37" t="n">
-        <v>19.3</v>
+        <v>19.4</v>
       </c>
       <c r="Y37" t="n">
         <v>-4</v>
@@ -9252,10 +9252,10 @@
         <v>0</v>
       </c>
       <c r="W38" t="n">
-        <v>5317</v>
+        <v>5418</v>
       </c>
       <c r="X38" t="n">
-        <v>12.4</v>
+        <v>12.7</v>
       </c>
       <c r="Y38" t="n">
         <v>26</v>
@@ -9484,7 +9484,7 @@
         <v>0.011</v>
       </c>
       <c r="W39" t="n">
-        <v>4183</v>
+        <v>4155</v>
       </c>
       <c r="X39" t="inlineStr"/>
       <c r="Y39" t="n">
@@ -9714,10 +9714,10 @@
         <v>0.114</v>
       </c>
       <c r="W40" t="n">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="X40" t="n">
-        <v>7.05</v>
+        <v>7.03</v>
       </c>
       <c r="Y40" t="n">
         <v>118</v>
@@ -10171,13 +10171,13 @@
         </is>
       </c>
       <c r="V42" t="n">
-        <v>0.131</v>
+        <v>0.138</v>
       </c>
       <c r="W42" t="n">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="X42" t="n">
-        <v>35.5</v>
+        <v>33.8</v>
       </c>
       <c r="Y42" t="n">
         <v>19</v>
@@ -10403,13 +10403,13 @@
         </is>
       </c>
       <c r="V43" t="n">
-        <v>0.099</v>
+        <v>0.1</v>
       </c>
       <c r="W43" t="n">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="X43" t="n">
-        <v>27.6</v>
+        <v>27.5</v>
       </c>
       <c r="Y43" t="n">
         <v>24</v>
@@ -10635,10 +10635,10 @@
         </is>
       </c>
       <c r="V44" t="n">
-        <v>0.053</v>
+        <v>0.052</v>
       </c>
       <c r="W44" t="n">
-        <v>938</v>
+        <v>944</v>
       </c>
       <c r="X44" t="inlineStr"/>
       <c r="Y44" t="n">
@@ -10868,10 +10868,10 @@
         <v>0</v>
       </c>
       <c r="W45" t="n">
-        <v>3830</v>
+        <v>3902</v>
       </c>
       <c r="X45" t="n">
-        <v>86.2</v>
+        <v>87.8</v>
       </c>
       <c r="Y45" t="n">
         <v>42</v>
@@ -11100,10 +11100,10 @@
         <v>0.006</v>
       </c>
       <c r="W46" t="n">
-        <v>4843</v>
+        <v>4898</v>
       </c>
       <c r="X46" t="n">
-        <v>12.5</v>
+        <v>12.7</v>
       </c>
       <c r="Y46" t="n">
         <v>23</v>
@@ -11328,10 +11328,10 @@
         <v>0</v>
       </c>
       <c r="W47" t="n">
-        <v>110771</v>
+        <v>108435</v>
       </c>
       <c r="X47" t="n">
-        <v>31.9</v>
+        <v>31.2</v>
       </c>
       <c r="Y47" t="n">
         <v>18</v>
@@ -11557,13 +11557,13 @@
         </is>
       </c>
       <c r="V48" t="n">
-        <v>0.218</v>
+        <v>0.217</v>
       </c>
       <c r="W48" t="n">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="X48" t="n">
-        <v>24.5</v>
+        <v>24.6</v>
       </c>
       <c r="Y48" t="n">
         <v>21</v>

</xml_diff>